<commit_message>
auto: snapshot 2026-09-14 13:31:01
</commit_message>
<xml_diff>
--- a/clan_3094.xlsx
+++ b/clan_3094.xlsx
@@ -51170,7 +51170,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-14 13:01:00</t>
+          <t>Timestamp: 2026-09-14 13:31:00</t>
         </is>
       </c>
     </row>
@@ -51213,11 +51213,11 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>7825</v>
+        <v>7870</v>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>+1850</t>
+          <t>+1895</t>
         </is>
       </c>
     </row>
@@ -51693,11 +51693,11 @@
         </is>
       </c>
       <c r="B37" s="5" t="n">
-        <v>9823</v>
+        <v>9873</v>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>+2287</t>
+          <t>+2337</t>
         </is>
       </c>
     </row>
@@ -51828,11 +51828,11 @@
         </is>
       </c>
       <c r="B46" s="5" t="n">
-        <v>9684</v>
+        <v>9734</v>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>+2305</t>
+          <t>+2355</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-15 13:31:01
</commit_message>
<xml_diff>
--- a/clan_3094.xlsx
+++ b/clan_3094.xlsx
@@ -52020,7 +52020,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-15 13:01:00</t>
+          <t>Timestamp: 2026-09-15 13:31:00</t>
         </is>
       </c>
     </row>
@@ -52078,11 +52078,11 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>6449</v>
+        <v>6499</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>+1003</t>
+          <t>+1053</t>
         </is>
       </c>
     </row>
@@ -52363,11 +52363,11 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>12092</v>
+        <v>12117</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>+1150</t>
+          <t>+1175</t>
         </is>
       </c>
     </row>
@@ -52393,11 +52393,11 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>6437</v>
+        <v>6487</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>+1050</t>
+          <t>+1100</t>
         </is>
       </c>
     </row>
@@ -52498,11 +52498,11 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>11466</v>
+        <v>11491</v>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>+1118</t>
+          <t>+1143</t>
         </is>
       </c>
     </row>
@@ -52513,11 +52513,11 @@
         </is>
       </c>
       <c r="B35" s="5" t="n">
-        <v>11456</v>
+        <v>11481</v>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>+1159</t>
+          <t>+1184</t>
         </is>
       </c>
     </row>
@@ -52528,11 +52528,11 @@
         </is>
       </c>
       <c r="B36" s="5" t="n">
-        <v>11311</v>
+        <v>11336</v>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>+1167</t>
+          <t>+1192</t>
         </is>
       </c>
     </row>
@@ -52543,11 +52543,11 @@
         </is>
       </c>
       <c r="B37" s="5" t="n">
-        <v>11036</v>
+        <v>11061</v>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>+1163</t>
+          <t>+1188</t>
         </is>
       </c>
     </row>
@@ -52678,11 +52678,11 @@
         </is>
       </c>
       <c r="B46" s="5" t="n">
-        <v>10877</v>
+        <v>10902</v>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>+1143</t>
+          <t>+1168</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-16 13:31:01
</commit_message>
<xml_diff>
--- a/clan_3094.xlsx
+++ b/clan_3094.xlsx
@@ -52870,7 +52870,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-16 13:01:00</t>
+          <t>Timestamp: 2026-09-16 13:31:00</t>
         </is>
       </c>
     </row>
@@ -52913,11 +52913,11 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>9312</v>
+        <v>9337</v>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>+629</t>
+          <t>+654</t>
         </is>
       </c>
     </row>
@@ -52928,11 +52928,11 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>7240</v>
+        <v>7265</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>+741</t>
+          <t>+766</t>
         </is>
       </c>
     </row>
@@ -52958,11 +52958,11 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>11397</v>
+        <v>11427</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>+325</t>
+          <t>+355</t>
         </is>
       </c>
     </row>
@@ -53123,11 +53123,11 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>11547</v>
+        <v>11597</v>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>+325</t>
+          <t>+375</t>
         </is>
       </c>
     </row>
@@ -53138,11 +53138,11 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>11484</v>
+        <v>11534</v>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>+313</t>
+          <t>+363</t>
         </is>
       </c>
     </row>
@@ -53153,11 +53153,11 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>11445</v>
+        <v>11495</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>+325</t>
+          <t>+375</t>
         </is>
       </c>
     </row>
@@ -53168,11 +53168,11 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>11155</v>
+        <v>11205</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>+297</t>
+          <t>+347</t>
         </is>
       </c>
     </row>
@@ -53183,11 +53183,11 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>11054</v>
+        <v>11104</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>+325</t>
+          <t>+375</t>
         </is>
       </c>
     </row>
@@ -53213,11 +53213,11 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>12845</v>
+        <v>12870</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>+728</t>
+          <t>+753</t>
         </is>
       </c>
     </row>
@@ -53243,11 +53243,11 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>7137</v>
+        <v>7162</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>+650</t>
+          <t>+675</t>
         </is>
       </c>
     </row>
@@ -53258,11 +53258,11 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>9791</v>
+        <v>9816</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>+575</t>
+          <t>+600</t>
         </is>
       </c>
     </row>
@@ -53273,11 +53273,11 @@
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>9543</v>
+        <v>9568</v>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>+575</t>
+          <t>+600</t>
         </is>
       </c>
     </row>
@@ -53288,11 +53288,11 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>9516</v>
+        <v>9541</v>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>+498</t>
+          <t>+523</t>
         </is>
       </c>
     </row>
@@ -53303,11 +53303,11 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>9662</v>
+        <v>9687</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>+650</t>
+          <t>+675</t>
         </is>
       </c>
     </row>
@@ -53318,11 +53318,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>9634</v>
+        <v>9659</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>+650</t>
+          <t>+675</t>
         </is>
       </c>
     </row>
@@ -53528,11 +53528,11 @@
         </is>
       </c>
       <c r="B46" s="5" t="n">
-        <v>11732</v>
+        <v>11766</v>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>+830</t>
+          <t>+864</t>
         </is>
       </c>
     </row>
@@ -53543,11 +53543,11 @@
         </is>
       </c>
       <c r="B47" s="5" t="n">
-        <v>9630</v>
+        <v>9680</v>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>+1344</t>
+          <t>+1394</t>
         </is>
       </c>
     </row>
@@ -53558,11 +53558,11 @@
         </is>
       </c>
       <c r="B48" s="5" t="n">
-        <v>10176</v>
+        <v>10226</v>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>+1890</t>
+          <t>+1940</t>
         </is>
       </c>
     </row>
@@ -53573,11 +53573,11 @@
         </is>
       </c>
       <c r="B49" s="5" t="n">
-        <v>8933</v>
+        <v>8983</v>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>+850</t>
+          <t>+900</t>
         </is>
       </c>
     </row>
@@ -53588,11 +53588,11 @@
         </is>
       </c>
       <c r="B50" s="5" t="n">
-        <v>9279</v>
+        <v>9297</v>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>+993</t>
+          <t>+1011</t>
         </is>
       </c>
     </row>
@@ -53663,11 +53663,11 @@
         </is>
       </c>
       <c r="B55" s="5" t="n">
-        <v>9129</v>
+        <v>9179</v>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>+843</t>
+          <t>+893</t>
         </is>
       </c>
     </row>
@@ -53678,11 +53678,11 @@
         </is>
       </c>
       <c r="B56" s="5" t="n">
-        <v>2408</v>
+        <v>2484</v>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+76</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-17 13:31:01
</commit_message>
<xml_diff>
--- a/clan_3094.xlsx
+++ b/clan_3094.xlsx
@@ -53720,7 +53720,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-17 13:01:00</t>
+          <t>Timestamp: 2026-09-17 13:31:00</t>
         </is>
       </c>
     </row>
@@ -54528,11 +54528,11 @@
         </is>
       </c>
       <c r="B56" s="5" t="n">
-        <v>2484</v>
+        <v>2584</v>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+100</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-18 13:31:01
</commit_message>
<xml_diff>
--- a/clan_3094.xlsx
+++ b/clan_3094.xlsx
@@ -54570,7 +54570,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-18 13:01:00</t>
+          <t>Timestamp: 2026-09-18 13:31:00</t>
         </is>
       </c>
     </row>
@@ -55243,11 +55243,11 @@
         </is>
       </c>
       <c r="B47" s="5" t="n">
-        <v>11013</v>
+        <v>11030</v>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>+1179</t>
+          <t>+1196</t>
         </is>
       </c>
     </row>
@@ -55258,11 +55258,11 @@
         </is>
       </c>
       <c r="B48" s="5" t="n">
-        <v>11466</v>
+        <v>11491</v>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>+1632</t>
+          <t>+1657</t>
         </is>
       </c>
     </row>
@@ -55273,11 +55273,11 @@
         </is>
       </c>
       <c r="B49" s="5" t="n">
-        <v>10248</v>
+        <v>10274</v>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>+655</t>
+          <t>+681</t>
         </is>
       </c>
     </row>
@@ -55288,11 +55288,11 @@
         </is>
       </c>
       <c r="B50" s="5" t="n">
-        <v>10590</v>
+        <v>10600</v>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>+756</t>
+          <t>+766</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-19 13:01:02
</commit_message>
<xml_diff>
--- a/clan_3094.xlsx
+++ b/clan_3094.xlsx
@@ -73,6 +73,7 @@
     <sheet name="2026-09-16" sheetId="64" state="visible" r:id="rId64"/>
     <sheet name="2026-09-17" sheetId="65" state="visible" r:id="rId65"/>
     <sheet name="2026-09-18" sheetId="66" state="visible" r:id="rId66"/>
+    <sheet name="2026-09-19" sheetId="67" state="visible" r:id="rId67"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -55395,6 +55396,855 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet67.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C56"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Sangre Latina Clan (3094)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-19 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Sebas</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>12446</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+512</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Kyara Senju™</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>11605</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+542</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Exe™</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>9635</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+696</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Ereshkigal</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>145</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>13694</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>+410</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Killua Senju™</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>10683</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+75</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Tsunade Senju™</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>10641</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>+75</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Mito Senju™</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>10602</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>+75</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Hisoka Senju™</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>10297</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+75</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Lambada</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>11288</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Orpheus</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>11451</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Ahrtheus</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>11177</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Euridice</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>11176</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Atenea</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>11014</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Persefone</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>10533</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>ll</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>13899</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+425</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>lll</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>13762</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+438</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>13815</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+422</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>13496</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+425</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>VI</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>13403</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+425</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Taylor Swift</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>1579</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>-121</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Himawari</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>14805</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+589</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Chrollo Senju™</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>10379</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+75</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Emily Chan™</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>9661</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+738</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drako </t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>12189</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+626</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Azusa Chan</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>11915</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>+572</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Arceus</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>11928</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+580</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fenraim </t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>11994</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+532</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Thurzin</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>11998</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+544</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Tamara Anbu</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>10927</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Yügao | Anbu</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>15003</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+698</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Hinoko | Anbu</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>15055</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>+694</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Kunoichi | Anbu</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>14855</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>+690</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Kaguya | Anbu</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>14567</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>+702</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Sabrina Carpenter</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>1563</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Haku Anbu</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>9770</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>+75</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Arch"</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>10467</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Kushina</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>10066</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Lucia</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>8567</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>+75</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Rosangel</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>2039</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Wisin y Yandel</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>1750</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Taylor Swift</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>1700</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Rö | Anbu</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>14495</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>+754</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>11965</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>+1381</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>12438</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>+1854</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>....</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>11144</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>+870</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>11439</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>+855</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>^^Radahn</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>4592</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>+275</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Zheninjas</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>Jounin Gakure</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>Bicho</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>4179</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>+267</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>11433</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>+849</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>ShaToshi</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>2680</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>+96</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-19 13:31:01
</commit_message>
<xml_diff>
--- a/clan_3094.xlsx
+++ b/clan_3094.xlsx
@@ -55420,7 +55420,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-19 13:01:00</t>
+          <t>Timestamp: 2026-09-19 13:31:00</t>
         </is>
       </c>
     </row>
@@ -55463,11 +55463,11 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>11605</v>
+        <v>11646</v>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>+542</t>
+          <t>+583</t>
         </is>
       </c>
     </row>
@@ -55508,11 +55508,11 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>13694</v>
+        <v>13744</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>+410</t>
+          <t>+460</t>
         </is>
       </c>
     </row>
@@ -55673,11 +55673,11 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>13899</v>
+        <v>13949</v>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>+425</t>
+          <t>+475</t>
         </is>
       </c>
     </row>
@@ -55688,11 +55688,11 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>13762</v>
+        <v>13812</v>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>+438</t>
+          <t>+488</t>
         </is>
       </c>
     </row>
@@ -55703,11 +55703,11 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>13815</v>
+        <v>13856</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>+422</t>
+          <t>+463</t>
         </is>
       </c>
     </row>
@@ -55718,11 +55718,11 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>13496</v>
+        <v>13546</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>+425</t>
+          <t>+475</t>
         </is>
       </c>
     </row>
@@ -55733,11 +55733,11 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>13403</v>
+        <v>13453</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>+425</t>
+          <t>+475</t>
         </is>
       </c>
     </row>
@@ -55808,11 +55808,11 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>12189</v>
+        <v>12239</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>+626</t>
+          <t>+676</t>
         </is>
       </c>
     </row>
@@ -55823,11 +55823,11 @@
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>11915</v>
+        <v>11965</v>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>+572</t>
+          <t>+622</t>
         </is>
       </c>
     </row>
@@ -55838,11 +55838,11 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>11928</v>
+        <v>11978</v>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>+580</t>
+          <t>+630</t>
         </is>
       </c>
     </row>
@@ -55853,11 +55853,11 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>11994</v>
+        <v>12044</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>+532</t>
+          <t>+582</t>
         </is>
       </c>
     </row>
@@ -55868,11 +55868,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>11998</v>
+        <v>12048</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>+544</t>
+          <t>+594</t>
         </is>
       </c>
     </row>

</xml_diff>